<commit_message>
Match capacitors to the schematic (add 100 nF), add vector schematic PDF, ignore KiCad local files
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SnnjAyMwjQGxr5nzvAhxEy
</commit_message>
<xml_diff>
--- a/BOM/ChromaSense_BOM_v2.xlsx
+++ b/BOM/ChromaSense_BOM_v2.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4200" yWindow="4200" windowWidth="28800" windowHeight="15225" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,8 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.00&quot; €&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0.000&quot; €&quot;"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -162,7 +163,9 @@
       <top style="thin">
         <color rgb="FFCCCCCC"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -171,9 +174,7 @@
       <top style="thin">
         <color rgb="FFCCCCCC"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -181,7 +182,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -220,25 +221,29 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -499,35 +504,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="10"/>
+    <col width="4" customWidth="1" style="17" min="1" max="1"/>
+    <col width="36" customWidth="1" style="17" min="2" max="2"/>
+    <col width="22" customWidth="1" style="17" min="3" max="3"/>
+    <col width="6" customWidth="1" style="17" min="4" max="4"/>
+    <col width="14" customWidth="1" style="17" min="5" max="5"/>
+    <col width="12" customWidth="1" style="17" min="6" max="6"/>
+    <col width="20" customWidth="1" style="17" min="7" max="7"/>
+    <col width="45" customWidth="1" style="17" min="8" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+    <row r="1" ht="36" customHeight="1" s="17">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>ChromaSense — Bill of Materials</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="19.5" customHeight="1" s="17">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>Project: Remote Color Sensor  |  OTH Regensburg — Faculty ANK  |  Supervisor: Prof. Johannes Wild</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="7.5" customHeight="1"/>
-    <row r="4" ht="21.75" customHeight="1">
+    <row r="3" ht="7.5" customHeight="1" s="17"/>
+    <row r="4" ht="21.75" customHeight="1" s="17">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>#</t>
@@ -579,7 +584,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="39.75" customHeight="1">
+    <row r="5" ht="39.75" customHeight="1" s="17">
       <c r="A5" s="2" t="n">
         <v>1</v>
       </c>
@@ -625,7 +630,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="39.75" customHeight="1">
+    <row r="6" ht="39.75" customHeight="1" s="17">
       <c r="A6" s="6" t="n">
         <v>2</v>
       </c>
@@ -671,7 +676,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="39.75" customHeight="1">
+    <row r="7" ht="39.75" customHeight="1" s="17">
       <c r="A7" s="2" t="n">
         <v>3</v>
       </c>
@@ -717,7 +722,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="39.75" customHeight="1">
+    <row r="8" ht="39.75" customHeight="1" s="17">
       <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
@@ -763,26 +768,26 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="39.75" customHeight="1">
+    <row r="9" ht="39.75" customHeight="1" s="17">
       <c r="A9" s="2" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Grove HY2.0-4P Connector
-I²C interface to M5Stack Core2</t>
+          <t>MLCC 100 nF / 16 V / X7R / 0402
+Decoupling capacitor (1.8 V rail)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>HY2.0-4P (SMD)</t>
+          <t>GRM155R71C104KA88D</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>0.35</v>
+        <v>100</v>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>0.005</v>
       </c>
       <c r="F9" s="4">
         <f>D9*E9</f>
@@ -790,45 +795,37 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Eckstein / Berrybase / M5Stack</t>
+          <t>LCSC</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>https://eckstein-shop.de/M5Stack-Grove-to-4-Pin-Connector-10pcs-EN</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>https://www.berrybase.de/m5stack-connector-grove-to-4-pin-10-stueck</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="inlineStr">
-        <is>
-          <t>https://docs.m5stack.com/en/module/extport_for_core2</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="39.75" customHeight="1">
+          <t>https://www.lcsc.com/product-detail/C71629.html</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="15" t="n"/>
+    </row>
+    <row r="10" ht="39.75" customHeight="1" s="17">
       <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>M5Stack Core2
-ESP32 IoT Development Kit (compute + display + battery platform)</t>
+          <t>Grove HY2.0-4P Connector
+I²C interface to M5Stack Core2</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>M5Stack Core2 v1.1</t>
+          <t>HY2.0-4P (SMD)</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>50</v>
+        <v>0.35</v>
       </c>
       <c r="F10" s="8">
         <f>D10*E10</f>
@@ -836,41 +833,45 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>M5Stack (official)</t>
+          <t>Eckstein / Berrybase / M5Stack</t>
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>https://shop.m5stack.com/products/m5stack-core2-esp32-iot-development-kit</t>
+          <t>https://eckstein-shop.de/M5Stack-Grove-to-4-Pin-Connector-10pcs-EN</t>
         </is>
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>https://docs.m5stack.com/en/core/core2</t>
-        </is>
-      </c>
-      <c r="J10" s="18" t="n"/>
-    </row>
-    <row r="11" ht="39.75" customHeight="1">
+          <t>https://www.berrybase.de/m5stack-connector-grove-to-4-pin-10-stueck</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>https://docs.m5stack.com/en/module/extport_for_core2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="39.75" customHeight="1" s="17">
       <c r="A11" s="2" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>PCB Fabrication — ChromaSense Breakout
-2-layer, 25×30 mm, 5 pcs, DRC clean, incl. shipping</t>
+          <t>M5Stack Core2
+ESP32 IoT Development Kit (compute + display + battery platform)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>JLCPCB 2-layer PCB</t>
+          <t>M5Stack Core2 v1.1</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="F11" s="4">
         <f>D11*E11</f>
@@ -878,45 +879,89 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
+          <t>M5Stack (official)</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>https://shop.m5stack.com/products/m5stack-core2-esp32-iot-development-kit</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>https://docs.m5stack.com/en/core/core2</t>
+        </is>
+      </c>
+      <c r="J11" s="15" t="n"/>
+    </row>
+    <row r="12" ht="39.75" customHeight="1" s="17">
+      <c r="A12" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>PCB Fabrication — ChromaSense Breakout
+2-layer, 25×30 mm, 5 pcs, DRC clean, incl. shipping</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>JLCPCB 2-layer PCB</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="8">
+        <f>D12*E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
           <t>JLCPCB</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>https://jlcpcb.com/</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="19" t="n"/>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="I12" s="9" t="n"/>
+      <c r="J12" s="14" t="n"/>
+    </row>
+    <row r="13" ht="36" customHeight="1" s="17">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>ESTIMATED TOTAL (excl. shipping)</t>
         </is>
       </c>
-      <c r="B12" s="20" t="n"/>
-      <c r="C12" s="20" t="n"/>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="10">
-        <f>SUM(F5:F11)</f>
+      <c r="B13" s="19" t="n"/>
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="19" t="n"/>
+      <c r="F13" s="10">
+        <f>SUM(F5:F12)</f>
         <v/>
       </c>
-      <c r="G12" s="11" t="n"/>
-      <c r="H12" s="11" t="n"/>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="11" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="17" t="n"/>
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="11" t="n"/>
+      <c r="I13" s="11" t="n"/>
+      <c r="J13" s="11" t="n"/>
+    </row>
+    <row r="14" s="17"/>
+    <row r="15" s="17"/>
+    <row r="16" s="17">
+      <c r="A16" s="16" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A12:E12"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A16:I16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId1"/>

</xml_diff>